<commit_message>
fix: barrett paper year from 2026 to 2016
</commit_message>
<xml_diff>
--- a/materials/25_random_scenario_judgement_rujuta.xlsx
+++ b/materials/25_random_scenario_judgement_rujuta.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1619" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1619" uniqueCount="362">
   <si>
     <t>paper_id</t>
   </si>
@@ -67,7 +67,7 @@
     <t>Objective/HO: ceding of substantial control, no intent stated. Access: decision authority delegated.</t>
   </si>
   <si>
-    <t>barrett_2026</t>
+    <t>barrett_2016</t>
   </si>
   <si>
     <t>S8</t>
@@ -371,6 +371,9 @@
   </si>
   <si>
     <t>Target: Gives only 'firms'; misses the human oversight given up.</t>
+  </si>
+  <si>
+    <t>barrett_2026</t>
   </si>
   <si>
     <t>Neuromorphic AI is seed AI</t>
@@ -2624,19 +2627,19 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>110</v>
@@ -2654,13 +2657,13 @@
         <v>115</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -2671,13 +2674,13 @@
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>110</v>
@@ -2685,7 +2688,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="4"/>
       <c r="I4" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>110</v>
@@ -2693,13 +2696,13 @@
       <c r="K4" s="2"/>
       <c r="L4" s="4"/>
       <c r="M4" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>110</v>
@@ -2720,7 +2723,7 @@
         <v>110</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>110</v>
@@ -2732,13 +2735,13 @@
       <c r="K5" s="2"/>
       <c r="L5" s="4"/>
       <c r="M5" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>110</v>
@@ -2753,19 +2756,19 @@
         <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>110</v>
@@ -2775,7 +2778,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="4"/>
       <c r="M6" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>110</v>
@@ -2787,7 +2790,7 @@
         <v>115</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -2798,19 +2801,19 @@
         <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>115</v>
@@ -2820,19 +2823,19 @@
       <c r="K7" s="2"/>
       <c r="L7" s="4"/>
       <c r="M7" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -2843,19 +2846,19 @@
         <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>110</v>
@@ -2867,7 +2870,7 @@
       <c r="M8" s="2"/>
       <c r="N8" s="4"/>
       <c r="O8" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>110</v>
@@ -2882,19 +2885,19 @@
         <v>30</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>110</v>
@@ -2902,19 +2905,19 @@
       <c r="I9" s="2"/>
       <c r="J9" s="4"/>
       <c r="K9" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>110</v>
@@ -2929,19 +2932,19 @@
         <v>30</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>110</v>
@@ -2949,25 +2952,25 @@
       <c r="I10" s="2"/>
       <c r="J10" s="4"/>
       <c r="K10" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>115</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
@@ -2978,19 +2981,19 @@
         <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>110</v>
@@ -2998,19 +3001,19 @@
       <c r="I11" s="2"/>
       <c r="J11" s="4"/>
       <c r="K11" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>110</v>
@@ -3025,7 +3028,7 @@
         <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>110</v>
@@ -3033,7 +3036,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="4"/>
       <c r="G12" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>110</v>
@@ -3043,7 +3046,7 @@
       <c r="K12" s="2"/>
       <c r="L12" s="4"/>
       <c r="M12" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>110</v>
@@ -3055,7 +3058,7 @@
         <v>115</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
@@ -3066,19 +3069,19 @@
         <v>30</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>110</v>
@@ -3088,13 +3091,13 @@
       <c r="K13" s="2"/>
       <c r="L13" s="4"/>
       <c r="M13" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>110</v>
@@ -3121,7 +3124,7 @@
         <v>115</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>110</v>
@@ -3129,13 +3132,13 @@
       <c r="I14" s="2"/>
       <c r="J14" s="4"/>
       <c r="K14" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>110</v>
@@ -3143,7 +3146,7 @@
       <c r="O14" s="2"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
@@ -3154,19 +3157,19 @@
         <v>34</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>110</v>
@@ -3178,7 +3181,7 @@
       <c r="M15" s="2"/>
       <c r="N15" s="4"/>
       <c r="O15" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>110</v>
@@ -3193,19 +3196,19 @@
         <v>12</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>110</v>
@@ -3213,19 +3216,19 @@
       <c r="I16" s="2"/>
       <c r="J16" s="4"/>
       <c r="K16" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>110</v>
@@ -3240,43 +3243,43 @@
         <v>34</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>110</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>110</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>110</v>
@@ -3291,49 +3294,49 @@
         <v>18</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>110</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>115</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
@@ -3344,19 +3347,19 @@
         <v>30</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>110</v>
@@ -3379,13 +3382,13 @@
         <v>34</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>110</v>
@@ -3407,13 +3410,13 @@
         <v>115</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
@@ -3424,43 +3427,43 @@
         <v>30</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>110</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>110</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>110</v>
@@ -3475,19 +3478,19 @@
         <v>30</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>110</v>
@@ -3495,25 +3498,25 @@
       <c r="I22" s="2"/>
       <c r="J22" s="4"/>
       <c r="K22" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>115</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
@@ -3524,13 +3527,13 @@
         <v>34</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>110</v>
@@ -3548,13 +3551,13 @@
         <v>115</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
@@ -3565,19 +3568,19 @@
         <v>30</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>110</v>
@@ -3587,19 +3590,19 @@
       <c r="K24" s="2"/>
       <c r="L24" s="4"/>
       <c r="M24" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="N24" s="5" t="s">
         <v>115</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q24" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -3610,19 +3613,19 @@
         <v>26</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>110</v>
@@ -3634,25 +3637,25 @@
         <v>115</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>110</v>
       </c>
       <c r="M25" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="O25" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="N25" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="P25" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -3663,19 +3666,19 @@
         <v>34</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>110</v>
@@ -3687,25 +3690,25 @@
         <v>115</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L26" s="5" t="s">
         <v>115</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N26" s="3" t="s">
         <v>110</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>110</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -3738,43 +3741,43 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>95</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>97</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>99</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>101</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>103</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>105</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>107</v>
@@ -3845,7 +3848,7 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
@@ -3893,7 +3896,7 @@
         <v>21</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -4052,7 +4055,7 @@
         <v>32</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -4107,7 +4110,7 @@
         <v>36</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -4270,7 +4273,7 @@
         <v>45</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -4378,7 +4381,7 @@
         <v>51</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -4486,7 +4489,7 @@
         <v>57</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -4708,7 +4711,7 @@
         <v>69</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -4812,7 +4815,7 @@
         <v>75</v>
       </c>
       <c r="S20" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -4926,7 +4929,7 @@
         <v>81</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
@@ -4979,7 +4982,7 @@
         <v>84</v>
       </c>
       <c r="S23" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -5034,7 +5037,7 @@
         <v>87</v>
       </c>
       <c r="S24" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
@@ -5093,7 +5096,7 @@
         <v>90</v>
       </c>
       <c r="S25" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
@@ -5152,7 +5155,7 @@
         <v>93</v>
       </c>
       <c r="S26" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -5184,34 +5187,34 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="N1" s="6" t="s">
         <v>10</v>
@@ -5241,10 +5244,10 @@
         <v>108</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
@@ -5258,13 +5261,13 @@
         <v>13</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>14</v>
@@ -5317,7 +5320,7 @@
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>18</v>
@@ -5326,13 +5329,13 @@
         <v>19</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>14</v>
@@ -5374,13 +5377,13 @@
         <v>110</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -5394,13 +5397,13 @@
         <v>23</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>14</v>
@@ -5445,10 +5448,10 @@
       </c>
       <c r="V4" s="2"/>
       <c r="W4" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -5462,13 +5465,13 @@
         <v>27</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>14</v>
@@ -5511,10 +5514,10 @@
       </c>
       <c r="V5" s="2"/>
       <c r="W5" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="X5" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
@@ -5528,13 +5531,13 @@
         <v>31</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>14</v>
@@ -5578,13 +5581,13 @@
         <v>115</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
@@ -5598,13 +5601,13 @@
         <v>35</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>14</v>
@@ -5648,7 +5651,7 @@
         <v>110</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
@@ -5664,13 +5667,13 @@
         <v>38</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>14</v>
@@ -5726,13 +5729,13 @@
         <v>41</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>14</v>
@@ -5792,13 +5795,13 @@
         <v>44</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>14</v>
@@ -5844,7 +5847,7 @@
         <v>110</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
@@ -5860,13 +5863,13 @@
         <v>47</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>14</v>
@@ -5926,13 +5929,13 @@
         <v>50</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>14</v>
@@ -5974,13 +5977,13 @@
         <v>115</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
@@ -5994,13 +5997,13 @@
         <v>53</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>14</v>
@@ -6058,13 +6061,13 @@
         <v>56</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>14</v>
@@ -6108,13 +6111,13 @@
       </c>
       <c r="U14" s="4"/>
       <c r="V14" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
@@ -6128,13 +6131,13 @@
         <v>59</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>14</v>
@@ -6190,13 +6193,13 @@
         <v>62</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>14</v>
@@ -6243,10 +6246,10 @@
       </c>
       <c r="V16" s="2"/>
       <c r="W16" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="X16" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
@@ -6260,13 +6263,13 @@
         <v>65</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>14</v>
@@ -6328,13 +6331,13 @@
         <v>68</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>14</v>
@@ -6382,7 +6385,7 @@
         <v>110</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
@@ -6398,13 +6401,13 @@
         <v>71</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>14</v>
@@ -6445,10 +6448,10 @@
       <c r="U19" s="4"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="X19" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
@@ -6462,13 +6465,13 @@
         <v>74</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>14</v>
@@ -6512,13 +6515,13 @@
         <v>110</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="W20" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="X20" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
@@ -6532,13 +6535,13 @@
         <v>77</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>14</v>
@@ -6600,13 +6603,13 @@
         <v>80</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>14</v>
@@ -6652,7 +6655,7 @@
         <v>110</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="W22" s="2"/>
       <c r="X22" s="2"/>
@@ -6668,13 +6671,13 @@
         <v>83</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>14</v>
@@ -6716,13 +6719,13 @@
         <v>110</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="W23" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="X23" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
@@ -6736,13 +6739,13 @@
         <v>86</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>14</v>
@@ -6786,7 +6789,7 @@
         <v>110</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="W24" s="2"/>
       <c r="X24" s="2"/>
@@ -6802,13 +6805,13 @@
         <v>89</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>14</v>
@@ -6856,13 +6859,13 @@
         <v>110</v>
       </c>
       <c r="V25" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="W25" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="X25" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
@@ -6876,13 +6879,13 @@
         <v>92</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>14</v>
@@ -6930,13 +6933,13 @@
         <v>110</v>
       </c>
       <c r="V26" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="W26" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="X26" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>